<commit_message>
data: actualizar evidencias OPS
</commit_message>
<xml_diff>
--- a/exports/Resumen_Evidencias_OPS.xlsx
+++ b/exports/Resumen_Evidencias_OPS.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiendas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actividades" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tiendas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Actividades" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$9:$H$15</definedName>
@@ -231,14 +231,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -262,7 +262,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -292,8 +292,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -320,8 +320,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -344,7 +344,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -359,9 +359,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>

</xml_diff>

<commit_message>
Add files via upload (#2)
</commit_message>
<xml_diff>
--- a/exports/Resumen_Evidencias_OPS.xlsx
+++ b/exports/Resumen_Evidencias_OPS.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Tiendas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Actividades" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiendas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actividades" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$9:$H$15</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Resumen'!$A$1:$H$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tiendas'!$A$4:$I$76</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Tiendas'!$1:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actividades'!$A$4:$H$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actividades'!$A$4:$H$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -592,7 +592,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Centro Norte · Corte 31/08/2026 16:00</t>
+          <t>Centro Norte · Corte 31/08/2026 20:06</t>
         </is>
       </c>
     </row>
@@ -615,10 +615,10 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>599</v>
+        <v>521</v>
       </c>
       <c r="E6" s="5">
         <f>IFERROR(A6/(A6+C6),0)</f>
@@ -681,10 +681,10 @@
         <v>10</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="F10" s="9">
         <f>IFERROR(D10/(D10+E10),0)</f>
@@ -707,17 +707,17 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Yazmin Chabela</t>
+          <t>Veronica Garcia</t>
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E11" s="12" t="n">
-        <v>107</v>
+        <v>79</v>
       </c>
       <c r="F11" s="13">
         <f>IFERROR(D11/(D11+E11),0)</f>
@@ -740,14 +740,14 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Veronica Garcia</t>
+          <t>Yazmin Chabela</t>
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E12" s="8" t="n">
         <v>95</v>
@@ -773,17 +773,17 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Vanessa Carreño</t>
+          <t>Nancy Carolina</t>
         </is>
       </c>
       <c r="C13" s="11" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D13" s="11" t="n">
         <v>14</v>
       </c>
       <c r="E13" s="12" t="n">
-        <v>116</v>
+        <v>94</v>
       </c>
       <c r="F13" s="13">
         <f>IFERROR(D13/(D13+E13),0)</f>
@@ -806,17 +806,17 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Nancy Carolina</t>
+          <t>Vanessa Carreño</t>
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F14" s="9">
         <f>IFERROR(D14/(D14+E14),0)</f>
@@ -846,10 +846,10 @@
         <v>13</v>
       </c>
       <c r="D15" s="11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E15" s="12" t="n">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="F15" s="13">
         <f>IFERROR(D15/(D15+E15),0)</f>
@@ -924,7 +924,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Centro Norte · Corte 31/08/2026 16:00</t>
+          <t>Centro Norte · Corte 31/08/2026 20:06</t>
         </is>
       </c>
     </row>
@@ -995,10 +995,10 @@
         </is>
       </c>
       <c r="E5" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G5" s="13">
         <f>IFERROR(E5/(E5+F5),0)</f>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G6" s="9">
         <f>IFERROR(E6/(E6+F6),0)</f>
@@ -1078,7 +1078,7 @@
         <v>6</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G7" s="13">
         <f>IFERROR(E7/(E7+F7),0)</f>
@@ -1101,24 +1101,24 @@
       </c>
       <c r="B8" s="17" t="inlineStr">
         <is>
-          <t>38695</t>
+          <t>38894</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Cetram 4 Caminos</t>
+          <t>Galerias Perinorte</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Yazmin Chabela Guadarrama</t>
+          <t>Enrique Cesar Flores</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
         <v>5</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G8" s="9">
         <f>IFERROR(E8/(E8+F8),0)</f>
@@ -1141,12 +1141,12 @@
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>38401</t>
+          <t>38368</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>Coacalco</t>
+          <t>Luna Park</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -1158,7 +1158,7 @@
         <v>5</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G9" s="13">
         <f>IFERROR(E9/(E9+F9),0)</f>
@@ -1181,24 +1181,24 @@
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>38894</t>
+          <t>38561</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Galerias Perinorte</t>
+          <t>Parque Toreo</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Enrique Cesar Flores</t>
+          <t>Yazmin Chabela Guadarrama</t>
         </is>
       </c>
       <c r="E10" s="7" t="n">
         <v>5</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G10" s="9">
         <f>IFERROR(E10/(E10+F10),0)</f>
@@ -1221,21 +1221,21 @@
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>38333</t>
+          <t>38695</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>Izcalli Mega</t>
+          <t>Cetram 4 Caminos</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Enrique Cesar Flores</t>
+          <t>Yazmin Chabela Guadarrama</t>
         </is>
       </c>
       <c r="E11" s="11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F11" s="11" t="n">
         <v>5</v>
@@ -1261,12 +1261,12 @@
       </c>
       <c r="B12" s="17" t="inlineStr">
         <is>
-          <t>38368</t>
+          <t>38401</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Luna Park</t>
+          <t>Coacalco</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
@@ -1275,7 +1275,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>5</v>
@@ -1301,21 +1301,21 @@
       </c>
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>38561</t>
+          <t>38333</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>Parque Toreo</t>
+          <t>Izcalli Mega</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Yazmin Chabela Guadarrama</t>
+          <t>Enrique Cesar Flores</t>
         </is>
       </c>
       <c r="E13" s="11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F13" s="11" t="n">
         <v>5</v>
@@ -1358,7 +1358,7 @@
         <v>4</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G14" s="9">
         <f>IFERROR(E14/(E14+F14),0)</f>
@@ -1398,7 +1398,7 @@
         <v>3</v>
       </c>
       <c r="F15" s="11" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G15" s="13">
         <f>IFERROR(E15/(E15+F15),0)</f>
@@ -1438,7 +1438,7 @@
         <v>2</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G16" s="9">
         <f>IFERROR(E16/(E16+F16),0)</f>
@@ -1478,7 +1478,7 @@
         <v>2</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G17" s="13">
         <f>IFERROR(E17/(E17+F17),0)</f>
@@ -1518,7 +1518,7 @@
         <v>2</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G18" s="9">
         <f>IFERROR(E18/(E18+F18),0)</f>
@@ -1541,24 +1541,24 @@
       </c>
       <c r="B19" s="15" t="inlineStr">
         <is>
-          <t>38859</t>
+          <t>38924</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>Plaza Satelite II N1</t>
+          <t>Plaza Aeropuerto</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Yazmin Chabela Guadarrama</t>
+          <t>Veronica Garcia Ortega</t>
         </is>
       </c>
       <c r="E19" s="11" t="n">
         <v>2</v>
       </c>
       <c r="F19" s="11" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G19" s="13">
         <f>IFERROR(E19/(E19+F19),0)</f>
@@ -1581,12 +1581,12 @@
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>38475</t>
+          <t>38859</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Satelite Centro Civico</t>
+          <t>Plaza Satelite II N1</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
@@ -1598,7 +1598,7 @@
         <v>2</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G20" s="9">
         <f>IFERROR(E20/(E20+F20),0)</f>
@@ -1621,24 +1621,24 @@
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>38606</t>
+          <t>38475</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>TlalnepantlaCarso</t>
+          <t>Satelite Centro Civico</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>Nancy Carolina Rodriguez Medina</t>
+          <t>Yazmin Chabela Guadarrama</t>
         </is>
       </c>
       <c r="E21" s="11" t="n">
         <v>2</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G21" s="13">
         <f>IFERROR(E21/(E21+F21),0)</f>
@@ -1661,12 +1661,12 @@
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
-          <t>38374</t>
+          <t>38606</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>Valle Dorado</t>
+          <t>TlalnepantlaCarso</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
@@ -1678,7 +1678,7 @@
         <v>2</v>
       </c>
       <c r="F22" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G22" s="9">
         <f>IFERROR(E22/(E22+F22),0)</f>
@@ -1701,12 +1701,12 @@
       </c>
       <c r="B23" s="15" t="inlineStr">
         <is>
-          <t>38186</t>
+          <t>38374</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>Arboledas</t>
+          <t>Valle Dorado</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
@@ -1715,10 +1715,10 @@
         </is>
       </c>
       <c r="E23" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F23" s="11" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G23" s="13">
         <f>IFERROR(E23/(E23+F23),0)</f>
@@ -1741,24 +1741,24 @@
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>43043</t>
+          <t>38186</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>Atizapan</t>
+          <t>Arboledas</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>Yazmin Haydee Garcia Gonzalez</t>
+          <t>Nancy Carolina Rodriguez Medina</t>
         </is>
       </c>
       <c r="E24" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F24" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G24" s="9">
         <f>IFERROR(E24/(E24+F24),0)</f>
@@ -1781,12 +1781,12 @@
       </c>
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>38149</t>
+          <t>43043</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>Bellavista</t>
+          <t>Atizapan</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
@@ -1798,7 +1798,7 @@
         <v>1</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G25" s="13">
         <f>IFERROR(E25/(E25+F25),0)</f>
@@ -1821,24 +1821,24 @@
       </c>
       <c r="B26" s="17" t="inlineStr">
         <is>
-          <t>38930</t>
+          <t>38149</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>Blvd. Aeropuerto dt</t>
+          <t>Bellavista</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>Veronica Garcia Ortega</t>
+          <t>Yazmin Haydee Garcia Gonzalez</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G26" s="9">
         <f>IFERROR(E26/(E26+F26),0)</f>
@@ -1861,24 +1861,24 @@
       </c>
       <c r="B27" s="15" t="inlineStr">
         <is>
-          <t>38527</t>
+          <t>38930</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>Camarones</t>
+          <t>Blvd. Aeropuerto dt</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Vanessa Carreño Rios</t>
+          <t>Veronica Garcia Ortega</t>
         </is>
       </c>
       <c r="E27" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G27" s="13">
         <f>IFERROR(E27/(E27+F27),0)</f>
@@ -1901,24 +1901,24 @@
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>38837</t>
+          <t>38529</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>Centenario Azcapotzalco</t>
+          <t>Bosques de Aragon</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>Vanessa Carreño Rios</t>
+          <t>Veronica Garcia Ortega</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G28" s="9">
         <f>IFERROR(E28/(E28+F28),0)</f>
@@ -1941,24 +1941,24 @@
       </c>
       <c r="B29" s="15" t="inlineStr">
         <is>
-          <t>38394</t>
+          <t>38527</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>Centro Comercial Lomas Verdes</t>
+          <t>Camarones</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Yazmin Haydee Garcia Gonzalez</t>
+          <t>Vanessa Carreño Rios</t>
         </is>
       </c>
       <c r="E29" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G29" s="13">
         <f>IFERROR(E29/(E29+F29),0)</f>
@@ -1981,24 +1981,24 @@
       </c>
       <c r="B30" s="17" t="inlineStr">
         <is>
-          <t>38535</t>
+          <t>38837</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>City Center Esmeralda</t>
+          <t>Centenario Azcapotzalco</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>Yazmin Haydee Garcia Gonzalez</t>
+          <t>Vanessa Carreño Rios</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G30" s="9">
         <f>IFERROR(E30/(E30+F30),0)</f>
@@ -2021,24 +2021,24 @@
       </c>
       <c r="B31" s="15" t="inlineStr">
         <is>
-          <t>38197</t>
+          <t>38394</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>Echegaray</t>
+          <t>Centro Comercial Lomas Verdes</t>
         </is>
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
-          <t>Yazmin Chabela Guadarrama</t>
+          <t>Yazmin Haydee Garcia Gonzalez</t>
         </is>
       </c>
       <c r="E31" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G31" s="13">
         <f>IFERROR(E31/(E31+F31),0)</f>
@@ -2061,24 +2061,24 @@
       </c>
       <c r="B32" s="17" t="inlineStr">
         <is>
-          <t>38431</t>
+          <t>38535</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>Eduardo Molina</t>
+          <t>City Center Esmeralda</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>Veronica Garcia Ortega</t>
+          <t>Yazmin Haydee Garcia Gonzalez</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G32" s="9">
         <f>IFERROR(E32/(E32+F32),0)</f>
@@ -2101,12 +2101,12 @@
       </c>
       <c r="B33" s="15" t="inlineStr">
         <is>
-          <t>38458</t>
+          <t>38197</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
         <is>
-          <t>El Rosario</t>
+          <t>Echegaray</t>
         </is>
       </c>
       <c r="D33" s="12" t="inlineStr">
@@ -2118,7 +2118,7 @@
         <v>1</v>
       </c>
       <c r="F33" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G33" s="13">
         <f>IFERROR(E33/(E33+F33),0)</f>
@@ -2141,24 +2141,24 @@
       </c>
       <c r="B34" s="17" t="inlineStr">
         <is>
-          <t>38363</t>
+          <t>38431</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>Galerias Atizapan</t>
+          <t>Eduardo Molina</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>Yazmin Haydee Garcia Gonzalez</t>
+          <t>Veronica Garcia Ortega</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F34" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G34" s="9">
         <f>IFERROR(E34/(E34+F34),0)</f>
@@ -2181,12 +2181,12 @@
       </c>
       <c r="B35" s="15" t="inlineStr">
         <is>
-          <t>38770</t>
+          <t>38458</t>
         </is>
       </c>
       <c r="C35" s="12" t="inlineStr">
         <is>
-          <t>Gustavo Baz 29</t>
+          <t>El Rosario</t>
         </is>
       </c>
       <c r="D35" s="12" t="inlineStr">
@@ -2198,7 +2198,7 @@
         <v>1</v>
       </c>
       <c r="F35" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G35" s="13">
         <f>IFERROR(E35/(E35+F35),0)</f>
@@ -2221,24 +2221,24 @@
       </c>
       <c r="B36" s="17" t="inlineStr">
         <is>
-          <t>38661</t>
+          <t>38903</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>Jinetes</t>
+          <t>Encuentro Oceania</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>Nancy Carolina Rodriguez Medina</t>
+          <t>Veronica Garcia Ortega</t>
         </is>
       </c>
       <c r="E36" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F36" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G36" s="9">
         <f>IFERROR(E36/(E36+F36),0)</f>
@@ -2261,24 +2261,24 @@
       </c>
       <c r="B37" s="15" t="inlineStr">
         <is>
-          <t>38205</t>
+          <t>38995</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr">
         <is>
-          <t>Lindavista</t>
+          <t>Encuentro Oceania II</t>
         </is>
       </c>
       <c r="D37" s="12" t="inlineStr">
         <is>
-          <t>Vanessa Carreño Rios</t>
+          <t>Veronica Garcia Ortega</t>
         </is>
       </c>
       <c r="E37" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G37" s="13">
         <f>IFERROR(E37/(E37+F37),0)</f>
@@ -2301,24 +2301,24 @@
       </c>
       <c r="B38" s="17" t="inlineStr">
         <is>
-          <t>38207</t>
+          <t>38507</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>Lindavista II</t>
+          <t>Espacio Vista del Valle</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>Vanessa Carreño Rios</t>
+          <t>Yazmin Haydee Garcia Gonzalez</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F38" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G38" s="9">
         <f>IFERROR(E38/(E38+F38),0)</f>
@@ -2341,12 +2341,12 @@
       </c>
       <c r="B39" s="15" t="inlineStr">
         <is>
-          <t>38119</t>
+          <t>38363</t>
         </is>
       </c>
       <c r="C39" s="12" t="inlineStr">
         <is>
-          <t>Lomas Verdes</t>
+          <t>Galerias Atizapan</t>
         </is>
       </c>
       <c r="D39" s="12" t="inlineStr">
@@ -2358,7 +2358,7 @@
         <v>1</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G39" s="13">
         <f>IFERROR(E39/(E39+F39),0)</f>
@@ -2381,24 +2381,24 @@
       </c>
       <c r="B40" s="17" t="inlineStr">
         <is>
-          <t>38270</t>
+          <t>38770</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>Lomas Verdes II</t>
+          <t>Gustavo Baz 29</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr">
         <is>
-          <t>Yazmin Haydee Garcia Gonzalez</t>
+          <t>Yazmin Chabela Guadarrama</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F40" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G40" s="9">
         <f>IFERROR(E40/(E40+F40),0)</f>
@@ -2421,24 +2421,24 @@
       </c>
       <c r="B41" s="15" t="inlineStr">
         <is>
-          <t>38371</t>
+          <t>38230</t>
         </is>
       </c>
       <c r="C41" s="12" t="inlineStr">
         <is>
-          <t>Montevideo DT</t>
+          <t>ITEMS Edo de Mexico</t>
         </is>
       </c>
       <c r="D41" s="12" t="inlineStr">
         <is>
-          <t>Vanessa Carreño Rios</t>
+          <t>Nancy Carolina Rodriguez Medina</t>
         </is>
       </c>
       <c r="E41" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F41" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G41" s="13">
         <f>IFERROR(E41/(E41+F41),0)</f>
@@ -2461,24 +2461,24 @@
       </c>
       <c r="B42" s="17" t="inlineStr">
         <is>
-          <t>43111</t>
+          <t>38661</t>
         </is>
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>Montevideo Insurgentes</t>
+          <t>Jinetes</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">
         <is>
-          <t>Vanessa Carreño Rios</t>
+          <t>Nancy Carolina Rodriguez Medina</t>
         </is>
       </c>
       <c r="E42" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F42" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G42" s="9">
         <f>IFERROR(E42/(E42+F42),0)</f>
@@ -2501,24 +2501,24 @@
       </c>
       <c r="B43" s="15" t="inlineStr">
         <is>
-          <t>38674</t>
+          <t>38205</t>
         </is>
       </c>
       <c r="C43" s="12" t="inlineStr">
         <is>
-          <t>Mundo E</t>
+          <t>Lindavista</t>
         </is>
       </c>
       <c r="D43" s="12" t="inlineStr">
         <is>
-          <t>Nancy Carolina Rodriguez Medina</t>
+          <t>Vanessa Carreño Rios</t>
         </is>
       </c>
       <c r="E43" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F43" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G43" s="13">
         <f>IFERROR(E43/(E43+F43),0)</f>
@@ -2541,24 +2541,24 @@
       </c>
       <c r="B44" s="17" t="inlineStr">
         <is>
-          <t>38845</t>
+          <t>38207</t>
         </is>
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>Mundo E II</t>
+          <t>Lindavista II</t>
         </is>
       </c>
       <c r="D44" s="8" t="inlineStr">
         <is>
-          <t>Nancy Carolina Rodriguez Medina</t>
+          <t>Vanessa Carreño Rios</t>
         </is>
       </c>
       <c r="E44" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F44" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G44" s="9">
         <f>IFERROR(E44/(E44+F44),0)</f>
@@ -2581,24 +2581,24 @@
       </c>
       <c r="B45" s="15" t="inlineStr">
         <is>
-          <t>43195</t>
+          <t>38119</t>
         </is>
       </c>
       <c r="C45" s="12" t="inlineStr">
         <is>
-          <t>Parque Jadin kiosko</t>
+          <t>Lomas Verdes</t>
         </is>
       </c>
       <c r="D45" s="12" t="inlineStr">
         <is>
-          <t>Vanessa Carreño Rios</t>
+          <t>Yazmin Haydee Garcia Gonzalez</t>
         </is>
       </c>
       <c r="E45" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F45" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G45" s="13">
         <f>IFERROR(E45/(E45+F45),0)</f>
@@ -2621,24 +2621,24 @@
       </c>
       <c r="B46" s="17" t="inlineStr">
         <is>
-          <t>38937</t>
+          <t>38270</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>Parque Tepeyac Piso 1</t>
+          <t>Lomas Verdes II</t>
         </is>
       </c>
       <c r="D46" s="8" t="inlineStr">
         <is>
-          <t>Veronica Garcia Ortega</t>
+          <t>Yazmin Haydee Garcia Gonzalez</t>
         </is>
       </c>
       <c r="E46" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F46" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G46" s="9">
         <f>IFERROR(E46/(E46+F46),0)</f>
@@ -2661,24 +2661,24 @@
       </c>
       <c r="B47" s="15" t="inlineStr">
         <is>
-          <t>38965</t>
+          <t>38371</t>
         </is>
       </c>
       <c r="C47" s="12" t="inlineStr">
         <is>
-          <t>Parque Tepeyac Piso 2</t>
+          <t>Montevideo DT</t>
         </is>
       </c>
       <c r="D47" s="12" t="inlineStr">
         <is>
-          <t>Veronica Garcia Ortega</t>
+          <t>Vanessa Carreño Rios</t>
         </is>
       </c>
       <c r="E47" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F47" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G47" s="13">
         <f>IFERROR(E47/(E47+F47),0)</f>
@@ -2701,24 +2701,24 @@
       </c>
       <c r="B48" s="17" t="inlineStr">
         <is>
-          <t>38590</t>
+          <t>43111</t>
         </is>
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>Parque Toreo II</t>
+          <t>Montevideo Insurgentes</t>
         </is>
       </c>
       <c r="D48" s="8" t="inlineStr">
         <is>
-          <t>Yazmin Chabela Guadarrama</t>
+          <t>Vanessa Carreño Rios</t>
         </is>
       </c>
       <c r="E48" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F48" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G48" s="9">
         <f>IFERROR(E48/(E48+F48),0)</f>
@@ -2741,24 +2741,24 @@
       </c>
       <c r="B49" s="15" t="inlineStr">
         <is>
-          <t>38546</t>
+          <t>38674</t>
         </is>
       </c>
       <c r="C49" s="12" t="inlineStr">
         <is>
-          <t>Patio Claveria</t>
+          <t>Mundo E</t>
         </is>
       </c>
       <c r="D49" s="12" t="inlineStr">
         <is>
-          <t>Vanessa Carreño Rios</t>
+          <t>Nancy Carolina Rodriguez Medina</t>
         </is>
       </c>
       <c r="E49" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F49" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G49" s="13">
         <f>IFERROR(E49/(E49+F49),0)</f>
@@ -2781,24 +2781,24 @@
       </c>
       <c r="B50" s="17" t="inlineStr">
         <is>
-          <t>38677</t>
+          <t>38845</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>Patio la Raza</t>
+          <t>Mundo E II</t>
         </is>
       </c>
       <c r="D50" s="8" t="inlineStr">
         <is>
-          <t>Vanessa Carreño Rios</t>
+          <t>Nancy Carolina Rodriguez Medina</t>
         </is>
       </c>
       <c r="E50" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F50" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G50" s="9">
         <f>IFERROR(E50/(E50+F50),0)</f>
@@ -2821,24 +2821,24 @@
       </c>
       <c r="B51" s="15" t="inlineStr">
         <is>
-          <t>38176</t>
+          <t>43195</t>
         </is>
       </c>
       <c r="C51" s="12" t="inlineStr">
         <is>
-          <t>Periferico Satélite DT</t>
+          <t>Parque Jadin kiosko</t>
         </is>
       </c>
       <c r="D51" s="12" t="inlineStr">
         <is>
-          <t>Yazmin Chabela Guadarrama</t>
+          <t>Vanessa Carreño Rios</t>
         </is>
       </c>
       <c r="E51" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F51" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G51" s="13">
         <f>IFERROR(E51/(E51+F51),0)</f>
@@ -2861,12 +2861,12 @@
       </c>
       <c r="B52" s="17" t="inlineStr">
         <is>
-          <t>38924</t>
+          <t>38937</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t>Plaza Aeropuerto</t>
+          <t>Parque Tepeyac Piso 1</t>
         </is>
       </c>
       <c r="D52" s="8" t="inlineStr">
@@ -2878,7 +2878,7 @@
         <v>1</v>
       </c>
       <c r="F52" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G52" s="9">
         <f>IFERROR(E52/(E52+F52),0)</f>
@@ -2901,24 +2901,24 @@
       </c>
       <c r="B53" s="15" t="inlineStr">
         <is>
-          <t>38427</t>
+          <t>38965</t>
         </is>
       </c>
       <c r="C53" s="12" t="inlineStr">
         <is>
-          <t>Plaza Satelite</t>
+          <t>Parque Tepeyac Piso 2</t>
         </is>
       </c>
       <c r="D53" s="12" t="inlineStr">
         <is>
-          <t>Yazmin Chabela Guadarrama</t>
+          <t>Veronica Garcia Ortega</t>
         </is>
       </c>
       <c r="E53" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F53" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G53" s="13">
         <f>IFERROR(E53/(E53+F53),0)</f>
@@ -2941,24 +2941,24 @@
       </c>
       <c r="B54" s="17" t="inlineStr">
         <is>
-          <t>38811</t>
+          <t>38590</t>
         </is>
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t>Plaza Tepeyac</t>
+          <t>Parque Toreo II</t>
         </is>
       </c>
       <c r="D54" s="8" t="inlineStr">
         <is>
-          <t>Veronica Garcia Ortega</t>
+          <t>Yazmin Chabela Guadarrama</t>
         </is>
       </c>
       <c r="E54" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F54" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G54" s="9">
         <f>IFERROR(E54/(E54+F54),0)</f>
@@ -2981,24 +2981,24 @@
       </c>
       <c r="B55" s="15" t="inlineStr">
         <is>
-          <t>43132</t>
+          <t>38792</t>
         </is>
       </c>
       <c r="C55" s="12" t="inlineStr">
         <is>
-          <t>Plaza Vista Norte</t>
+          <t>Pasaje Tlanepantla</t>
         </is>
       </c>
       <c r="D55" s="12" t="inlineStr">
         <is>
-          <t>Vanessa Carreño Rios</t>
+          <t>Nancy Carolina Rodriguez Medina</t>
         </is>
       </c>
       <c r="E55" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F55" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G55" s="13">
         <f>IFERROR(E55/(E55+F55),0)</f>
@@ -3021,24 +3021,24 @@
       </c>
       <c r="B56" s="17" t="inlineStr">
         <is>
-          <t>38136</t>
+          <t>38546</t>
         </is>
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t>Punta Norte</t>
+          <t>Patio Claveria</t>
         </is>
       </c>
       <c r="D56" s="8" t="inlineStr">
         <is>
-          <t>Nancy Carolina Rodriguez Medina</t>
+          <t>Vanessa Carreño Rios</t>
         </is>
       </c>
       <c r="E56" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F56" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G56" s="9">
         <f>IFERROR(E56/(E56+F56),0)</f>
@@ -3061,24 +3061,24 @@
       </c>
       <c r="B57" s="15" t="inlineStr">
         <is>
-          <t>43152</t>
+          <t>38677</t>
         </is>
       </c>
       <c r="C57" s="12" t="inlineStr">
         <is>
-          <t>Samara Satélite</t>
+          <t>Patio la Raza</t>
         </is>
       </c>
       <c r="D57" s="12" t="inlineStr">
         <is>
-          <t>Yazmin Chabela Guadarrama</t>
+          <t>Vanessa Carreño Rios</t>
         </is>
       </c>
       <c r="E57" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F57" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G57" s="13">
         <f>IFERROR(E57/(E57+F57),0)</f>
@@ -3101,24 +3101,24 @@
       </c>
       <c r="B58" s="17" t="inlineStr">
         <is>
-          <t>38266</t>
+          <t>38176</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t>San Mateo</t>
+          <t>Periferico Satélite DT</t>
         </is>
       </c>
       <c r="D58" s="8" t="inlineStr">
         <is>
-          <t>Yazmin Haydee Garcia Gonzalez</t>
+          <t>Yazmin Chabela Guadarrama</t>
         </is>
       </c>
       <c r="E58" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F58" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G58" s="9">
         <f>IFERROR(E58/(E58+F58),0)</f>
@@ -3141,24 +3141,24 @@
       </c>
       <c r="B59" s="15" t="inlineStr">
         <is>
-          <t>38460</t>
+          <t>38427</t>
         </is>
       </c>
       <c r="C59" s="12" t="inlineStr">
         <is>
-          <t>Santa Monica</t>
+          <t>Plaza Satelite</t>
         </is>
       </c>
       <c r="D59" s="12" t="inlineStr">
         <is>
-          <t>Nancy Carolina Rodriguez Medina</t>
+          <t>Yazmin Chabela Guadarrama</t>
         </is>
       </c>
       <c r="E59" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F59" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G59" s="13">
         <f>IFERROR(E59/(E59+F59),0)</f>
@@ -3181,24 +3181,24 @@
       </c>
       <c r="B60" s="17" t="inlineStr">
         <is>
-          <t>38117</t>
+          <t>38811</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t>Satelite</t>
+          <t>Plaza Tepeyac</t>
         </is>
       </c>
       <c r="D60" s="8" t="inlineStr">
         <is>
-          <t>Yazmin Chabela Guadarrama</t>
+          <t>Veronica Garcia Ortega</t>
         </is>
       </c>
       <c r="E60" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F60" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G60" s="9">
         <f>IFERROR(E60/(E60+F60),0)</f>
@@ -3221,24 +3221,24 @@
       </c>
       <c r="B61" s="15" t="inlineStr">
         <is>
-          <t>38442</t>
+          <t>43132</t>
         </is>
       </c>
       <c r="C61" s="12" t="inlineStr">
         <is>
-          <t>Sor Juana</t>
+          <t>Plaza Vista Norte</t>
         </is>
       </c>
       <c r="D61" s="12" t="inlineStr">
         <is>
-          <t>Nancy Carolina Rodriguez Medina</t>
+          <t>Vanessa Carreño Rios</t>
         </is>
       </c>
       <c r="E61" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F61" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G61" s="13">
         <f>IFERROR(E61/(E61+F61),0)</f>
@@ -3261,24 +3261,24 @@
       </c>
       <c r="B62" s="17" t="inlineStr">
         <is>
-          <t>38925</t>
+          <t>38136</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
         <is>
-          <t>Star Medica Lomas Verdes</t>
+          <t>Punta Norte</t>
         </is>
       </c>
       <c r="D62" s="8" t="inlineStr">
         <is>
-          <t>Yazmin Haydee Garcia Gonzalez</t>
+          <t>Nancy Carolina Rodriguez Medina</t>
         </is>
       </c>
       <c r="E62" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F62" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G62" s="9">
         <f>IFERROR(E62/(E62+F62),0)</f>
@@ -3301,24 +3301,24 @@
       </c>
       <c r="B63" s="15" t="inlineStr">
         <is>
-          <t>38992</t>
+          <t>43152</t>
         </is>
       </c>
       <c r="C63" s="12" t="inlineStr">
         <is>
-          <t>Tapo Puerta Oriente</t>
+          <t>Samara Satélite</t>
         </is>
       </c>
       <c r="D63" s="12" t="inlineStr">
         <is>
-          <t>Veronica Garcia Ortega</t>
+          <t>Yazmin Chabela Guadarrama</t>
         </is>
       </c>
       <c r="E63" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F63" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G63" s="13">
         <f>IFERROR(E63/(E63+F63),0)</f>
@@ -3341,24 +3341,24 @@
       </c>
       <c r="B64" s="17" t="inlineStr">
         <is>
-          <t>38411</t>
+          <t>38266</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
         <is>
-          <t>Torres Lindavista</t>
+          <t>San Mateo</t>
         </is>
       </c>
       <c r="D64" s="8" t="inlineStr">
         <is>
-          <t>Vanessa Carreño Rios</t>
+          <t>Yazmin Haydee Garcia Gonzalez</t>
         </is>
       </c>
       <c r="E64" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F64" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G64" s="9">
         <f>IFERROR(E64/(E64+F64),0)</f>
@@ -3381,24 +3381,24 @@
       </c>
       <c r="B65" s="15" t="inlineStr">
         <is>
-          <t>43130</t>
+          <t>38460</t>
         </is>
       </c>
       <c r="C65" s="12" t="inlineStr">
         <is>
-          <t>Town Center Nicolás Romero</t>
+          <t>Santa Monica</t>
         </is>
       </c>
       <c r="D65" s="12" t="inlineStr">
         <is>
-          <t>Yazmin Haydee Garcia Gonzalez</t>
+          <t>Nancy Carolina Rodriguez Medina</t>
         </is>
       </c>
       <c r="E65" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F65" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G65" s="13">
         <f>IFERROR(E65/(E65+F65),0)</f>
@@ -3421,24 +3421,24 @@
       </c>
       <c r="B66" s="17" t="inlineStr">
         <is>
-          <t>38651</t>
+          <t>38117</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t>Via Vallejo</t>
+          <t>Satelite</t>
         </is>
       </c>
       <c r="D66" s="8" t="inlineStr">
         <is>
-          <t>Vanessa Carreño Rios</t>
+          <t>Yazmin Chabela Guadarrama</t>
         </is>
       </c>
       <c r="E66" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F66" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G66" s="9">
         <f>IFERROR(E66/(E66+F66),0)</f>
@@ -3461,12 +3461,12 @@
       </c>
       <c r="B67" s="15" t="inlineStr">
         <is>
-          <t>38694</t>
+          <t>38442</t>
         </is>
       </c>
       <c r="C67" s="12" t="inlineStr">
         <is>
-          <t>Villas de la Hacienda</t>
+          <t>Sor Juana</t>
         </is>
       </c>
       <c r="D67" s="12" t="inlineStr">
@@ -3478,7 +3478,7 @@
         <v>1</v>
       </c>
       <c r="F67" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G67" s="13">
         <f>IFERROR(E67/(E67+F67),0)</f>
@@ -3501,24 +3501,24 @@
       </c>
       <c r="B68" s="17" t="inlineStr">
         <is>
-          <t>38656</t>
+          <t>38925</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t>Viveros de la Loma</t>
+          <t>Star Medica Lomas Verdes</t>
         </is>
       </c>
       <c r="D68" s="8" t="inlineStr">
         <is>
-          <t>Yazmin Chabela Guadarrama</t>
+          <t>Yazmin Haydee Garcia Gonzalez</t>
         </is>
       </c>
       <c r="E68" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F68" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G68" s="9">
         <f>IFERROR(E68/(E68+F68),0)</f>
@@ -3541,24 +3541,24 @@
       </c>
       <c r="B69" s="15" t="inlineStr">
         <is>
-          <t>38115</t>
+          <t>38992</t>
         </is>
       </c>
       <c r="C69" s="12" t="inlineStr">
         <is>
-          <t>Zona Azul</t>
+          <t>Tapo Puerta Oriente</t>
         </is>
       </c>
       <c r="D69" s="12" t="inlineStr">
         <is>
-          <t>Yazmin Haydee Garcia Gonzalez</t>
+          <t>Veronica Garcia Ortega</t>
         </is>
       </c>
       <c r="E69" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F69" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G69" s="13">
         <f>IFERROR(E69/(E69+F69),0)</f>
@@ -3581,24 +3581,24 @@
       </c>
       <c r="B70" s="17" t="inlineStr">
         <is>
-          <t>38142</t>
+          <t>38411</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t>Zona Esmeralda</t>
+          <t>Torres Lindavista</t>
         </is>
       </c>
       <c r="D70" s="8" t="inlineStr">
         <is>
-          <t>Yazmin Haydee Garcia Gonzalez</t>
+          <t>Vanessa Carreño Rios</t>
         </is>
       </c>
       <c r="E70" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F70" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G70" s="9">
         <f>IFERROR(E70/(E70+F70),0)</f>
@@ -3621,24 +3621,24 @@
       </c>
       <c r="B71" s="15" t="inlineStr">
         <is>
-          <t>38529</t>
+          <t>43130</t>
         </is>
       </c>
       <c r="C71" s="12" t="inlineStr">
         <is>
-          <t>Bosques de Aragon</t>
+          <t>Town Center Nicolás Romero</t>
         </is>
       </c>
       <c r="D71" s="12" t="inlineStr">
         <is>
-          <t>Veronica Garcia Ortega</t>
+          <t>Yazmin Haydee Garcia Gonzalez</t>
         </is>
       </c>
       <c r="E71" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F71" s="11" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G71" s="13">
         <f>IFERROR(E71/(E71+F71),0)</f>
@@ -3661,24 +3661,24 @@
       </c>
       <c r="B72" s="17" t="inlineStr">
         <is>
-          <t>38903</t>
+          <t>38651</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t>Encuentro Oceania</t>
+          <t>Via Vallejo</t>
         </is>
       </c>
       <c r="D72" s="8" t="inlineStr">
         <is>
-          <t>Veronica Garcia Ortega</t>
+          <t>Vanessa Carreño Rios</t>
         </is>
       </c>
       <c r="E72" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F72" s="7" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G72" s="9">
         <f>IFERROR(E72/(E72+F72),0)</f>
@@ -3701,24 +3701,24 @@
       </c>
       <c r="B73" s="15" t="inlineStr">
         <is>
-          <t>38995</t>
+          <t>38694</t>
         </is>
       </c>
       <c r="C73" s="12" t="inlineStr">
         <is>
-          <t>Encuentro Oceania II</t>
+          <t>Villas de la Hacienda</t>
         </is>
       </c>
       <c r="D73" s="12" t="inlineStr">
         <is>
-          <t>Veronica Garcia Ortega</t>
+          <t>Nancy Carolina Rodriguez Medina</t>
         </is>
       </c>
       <c r="E73" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F73" s="11" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G73" s="13">
         <f>IFERROR(E73/(E73+F73),0)</f>
@@ -3741,24 +3741,24 @@
       </c>
       <c r="B74" s="17" t="inlineStr">
         <is>
-          <t>38507</t>
+          <t>38656</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t>Espacio Vista del Valle</t>
+          <t>Viveros de la Loma</t>
         </is>
       </c>
       <c r="D74" s="8" t="inlineStr">
         <is>
-          <t>Yazmin Haydee Garcia Gonzalez</t>
+          <t>Yazmin Chabela Guadarrama</t>
         </is>
       </c>
       <c r="E74" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F74" s="7" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G74" s="9">
         <f>IFERROR(E74/(E74+F74),0)</f>
@@ -3781,24 +3781,24 @@
       </c>
       <c r="B75" s="15" t="inlineStr">
         <is>
-          <t>38230</t>
+          <t>38115</t>
         </is>
       </c>
       <c r="C75" s="12" t="inlineStr">
         <is>
-          <t>ITEMS Edo de Mexico</t>
+          <t>Zona Azul</t>
         </is>
       </c>
       <c r="D75" s="12" t="inlineStr">
         <is>
-          <t>Nancy Carolina Rodriguez Medina</t>
+          <t>Yazmin Haydee Garcia Gonzalez</t>
         </is>
       </c>
       <c r="E75" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F75" s="11" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G75" s="13">
         <f>IFERROR(E75/(E75+F75),0)</f>
@@ -3821,24 +3821,24 @@
       </c>
       <c r="B76" s="17" t="inlineStr">
         <is>
-          <t>38792</t>
+          <t>38142</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t>Pasaje Tlanepantla</t>
+          <t>Zona Esmeralda</t>
         </is>
       </c>
       <c r="D76" s="8" t="inlineStr">
         <is>
-          <t>Nancy Carolina Rodriguez Medina</t>
+          <t>Yazmin Haydee Garcia Gonzalez</t>
         </is>
       </c>
       <c r="E76" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F76" s="7" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G76" s="9">
         <f>IFERROR(E76/(E76+F76),0)</f>
@@ -3882,7 +3882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3906,7 +3906,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Centro Norte · Corte 31/08/2026 16:00</t>
+          <t>Centro Norte · Corte 31/08/2026 20:06</t>
         </is>
       </c>
     </row>
@@ -4063,14 +4063,14 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>QR - Qualtrics</t>
+          <t>Max &amp; Min</t>
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E8" s="9">
         <f>IFERROR(C8/(C8+D8),0)</f>
@@ -4078,7 +4078,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>03/09/26</t>
+          <t>06/09/26</t>
         </is>
       </c>
       <c r="G8" s="14" t="inlineStr">
@@ -4098,14 +4098,14 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Max &amp; Min</t>
+          <t>Fotografia - SM</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D9" s="11" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E9" s="13">
         <f>IFERROR(C9/(C9+D9),0)</f>
@@ -4133,14 +4133,14 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Fotografia - SM</t>
+          <t>Mandil Verde</t>
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E10" s="9">
         <f>IFERROR(C10/(C10+D10),0)</f>
@@ -4148,7 +4148,7 @@
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>06/09/26</t>
+          <t>13/09/26</t>
         </is>
       </c>
       <c r="G10" s="14" t="inlineStr">
@@ -4168,7 +4168,7 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Mandil Verde</t>
+          <t>Lay Out</t>
         </is>
       </c>
       <c r="C11" s="11" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>13/09/26</t>
+          <t>06/09/26</t>
         </is>
       </c>
       <c r="G11" s="14" t="inlineStr">
@@ -4203,11 +4203,11 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Lay Out</t>
+          <t>Community Board</t>
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D12" s="7" t="n">
         <v>67</v>
@@ -4218,7 +4218,7 @@
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>06/09/26</t>
+          <t>03/09/26</t>
         </is>
       </c>
       <c r="G12" s="14" t="inlineStr">
@@ -4238,14 +4238,14 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Community Board</t>
+          <t>Activacion PSL Sharpie</t>
         </is>
       </c>
       <c r="C13" s="11" t="n">
-        <v>1</v>
+        <v>72</v>
       </c>
       <c r="D13" s="11" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="E13" s="13">
         <f>IFERROR(C13/(C13+D13),0)</f>
@@ -4253,62 +4253,27 @@
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>03/09/26</t>
-        </is>
-      </c>
-      <c r="G13" s="14" t="inlineStr">
-        <is>
-          <t>Atención</t>
-        </is>
-      </c>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>Priorizar hoy</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="21" customHeight="1">
-      <c r="A14" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Activacion PSL Sharpie</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="n">
-        <v>66</v>
-      </c>
-      <c r="D14" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="E14" s="9">
-        <f>IFERROR(C14/(C14+D14),0)</f>
-        <v/>
-      </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
           <t>31/08/26</t>
         </is>
       </c>
-      <c r="G14" s="16" t="inlineStr">
+      <c r="G13" s="16" t="inlineStr">
         <is>
           <t>En meta</t>
         </is>
       </c>
-      <c r="H14" s="16" t="inlineStr">
+      <c r="H13" s="16" t="inlineStr">
         <is>
           <t>Mantener estándar</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H14"/>
+  <autoFilter ref="A4:H13"/>
   <mergeCells count="2">
     <mergeCell ref="A1:H2"/>
     <mergeCell ref="A3:H3"/>
   </mergeCells>
-  <conditionalFormatting sqref="E5:E14">
+  <conditionalFormatting sqref="E5:E13">
     <cfRule type="dataBar" priority="1">
       <dataBar showValue="1">
         <cfvo type="num" val="0"/>

</xml_diff>